<commit_message>
v0.0.4 - code review fixes
- Remove hardcoded credentials from application.yaml (security)
- Fix NPE on non-string cells in ExcelProductImportSource
- Add null checks after WebClient.block() in AuthClientImpl and ImageClientImpl
- Remove dead detectProductColumn() and IMAGE_COLUMN from ExcelHyperlinkCatalogImpl
- Delete unused TestClass, ImageMatcher, HyperlinkFileStructure
- Clean up crop temp files after upload (ImageServiceImpl)
- Delete downloaded EXCEL_HYPERLINK temp images after import (ProductImportService)
- Upgrade log level for download failures: INFO -> WARN (ExcelHyperlinkImageProvider)
- Validate placeholder image exists at startup (PlaceholderImageProvider)
- Add explicit Content-Type: application/json to login request

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/input/missing-products/1.xlsx
+++ b/input/missing-products/1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\webuser_3\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C49C32-E033-400A-9B62-CD9D23B054D1}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2691B7E9-4362-4347-8287-BB9267663F15}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet" sheetId="1" r:id="rId1"/>
@@ -20,69 +20,90 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Message</t>
   </si>
   <si>
-    <t>Ячейка E35, Определение продукта роза крашеная черная планета не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E49, Определение продукта роза матча не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E164, Определение продукта роза ветвистая викториан классик nl не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E184, Определение продукта роза ветвистая пьяно красная nl не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E185, Определение продукта роза ветвистая резиденс nl не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E194, Определение продукта роза ветвистая сноуфлейк nl не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E195, Определение продукта роза ветвистая сноуфлейк nl не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E207, Определение продукта гвоздика мати сиреневая не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E211, Определение продукта питтоспорум ралфи не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E243, Определение продукта хризантема пингпонг розовая китай, шт не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E261, Определение продукта анигозантус зеленый не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E262, Определение продукта антиринум белый армения не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E263, Определение продукта антиринум желтый армения не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E264, Определение продукта антиринум красный армения не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E266, Определение продукта антиринум розовый армения не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E267, Определение продукта арункус не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E286, Определение продукта гербера светло-розовая не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E335, Определение продукта пион флоренс никольс не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E339, Определение продукта скабиоза стеллата не найдено или не связано с предоставленными складами</t>
-  </si>
-  <si>
-    <t>Ячейка E343, Определение продукта эрика розовая не найдено или не связано с предоставленными складами</t>
+    <t>Ячейка E149, Определение продукта роза беллевью не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E188, Определение продукта роза ветвистая азор nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E190, Определение продукта роза ветвистая бачелор nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E196, Определение продукта роза ветвистая вуетте nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E201, Определение продукта роза ветвистая дарлингтон nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E212, Определение продукта роза ветвистая нанди не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E222, Определение продукта роза ветвистая рубикон nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E225, Определение продукта роза ветвистая салинеро nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E226, Определение продукта роза ветвистая саммер дэнс nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E227, Определение продукта роза ветвистая саммер роуз nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E228, Определение продукта роза ветвистая сансет меджик nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E232, Определение продукта роза ветвистая сильвия пинк nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E243, Определение продукта роза ветвистая хэппи вейдинг nl не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E246, Определение продукта роза ветвистая ёрс энд фаер не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E264, Определение продукта гвоздика мини персиковая не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E315, Определение продукта антиринум сильвер не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E316, Определение продукта антуриум блэк лав не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E352, Определение продукта калла самур не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E353, Определение продукта калла эскейп не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E355, Определение продукта кампанула зелено-розовая не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E357, Определение продукта котинус не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E371, Определение продукта матиола лавандовая не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E375, Определение продукта мята, пуч не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E385, Определение продукта пион авис не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E386, Определение продукта пион аивори белый не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E395, Определение продукта ранункулюс белый тесса не найдено или не связано с предоставленными складами</t>
+  </si>
+  <si>
+    <t>Ячейка E396, Определение продукта ранункулюс ханой тесса не найдено или не связано с предоставленными складами</t>
   </si>
 </sst>
 </file>
@@ -434,8 +455,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="122.28515625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -542,6 +566,41 @@
         <v>20</v>
       </c>
     </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>